<commit_message>
DF-01 nghe: hiển thị tranh lựa chọn + đáp án dạng mô tả ở 11_DUYET, câu (2) nhóm hiện script/bài đọc chung, sửa nhiễu JQ-0051/0053; prompt nghe yêu cầu mô tả ①②③
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011epdNWjc77FA9dxPqBsa8Z
</commit_message>
<xml_diff>
--- a/exports/DF-01_media_checklist.xlsx
+++ b/exports/DF-01_media_checklist.xlsx
@@ -643,7 +643,7 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>Tranh minh hoạ phẳng, nét đen mảnh, màu pastel nhẹ, nền trắng, bối cảnh Nhật Bản, không có chữ. Ảnh gồm 3 khung ngang bằng nhau, đánh số 1, 2, 3 to rõ ở góc trên trái mỗi khung; cùng nhân vật, cùng phong cách, chỉ khác ở điểm được hỏi. Ba đồng hồ treo tường: (1) 10:00, (2) 1:00, (3) 11:00.</t>
+          <t>Tranh minh hoạ phẳng, nét đen mảnh, màu pastel nhẹ, nền trắng, bối cảnh Nhật Bản, không có chữ. Ảnh gồm 3 khung ngang bằng nhau, đánh số 1, 2, 3 to rõ ở góc trên trái mỗi khung; cùng nhân vật, cùng phong cách, chỉ khác ở điểm được hỏi. Ba đồng hồ treo tường giống nhau: (1) 10:00, (2) 10:30, (3) 11:00.</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>Tranh minh hoạ phẳng, nét đen mảnh, màu pastel nhẹ, nền trắng, bối cảnh Nhật Bản, không có chữ. Ảnh gồm 3 khung ngang bằng nhau, đánh số 1, 2, 3 to rõ ở góc trên trái mỗi khung; cùng nhân vật, cùng phong cách, chỉ khác ở điểm được hỏi. Khay đồ ăn: (1) hamburger và cốc nước ép, (2) hamburger và tách cà phê, (3) hamburger, khoai tây chiên và cà phê.</t>
+          <t>Tranh minh hoạ phẳng, nét đen mảnh, màu pastel nhẹ, nền trắng, bối cảnh Nhật Bản, không có chữ. Ảnh gồm 3 khung ngang bằng nhau, đánh số 1, 2, 3 to rõ ở góc trên trái mỗi khung; cùng nhân vật, cùng phong cách, chỉ khác ở điểm được hỏi. Khay đồ ăn: (1) hamburger + cốc nước ép cỡ vừa (M), (2) hamburger + tách cà phê, (3) hamburger + cốc nước ép cỡ nhỏ (S).</t>
         </is>
       </c>
     </row>

</xml_diff>